<commit_message>
Paper - File Update
</commit_message>
<xml_diff>
--- a/Data/Crosswalks/GLORIA-Eora26 - Crosswalk.xlsx
+++ b/Data/Crosswalks/GLORIA-Eora26 - Crosswalk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://randus-my.sharepoint.com/personal/festeves_rand_org/Documents/Courses/Dissertation/3rd Paper/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://randus-my.sharepoint.com/personal/festeves_rand_org/Documents/Courses/Dissertation/3rd Paper/Repos/SSP-employment_estimates/Data/Crosswalks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{FB9AA796-4231-4B2A-BBF6-6B844FD14C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6312796-252D-497C-8C09-120E4D891506}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{FB9AA796-4231-4B2A-BBF6-6B844FD14C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6DEC31E-473E-4662-8FD5-F3F4AFA5B7C6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{34119B0E-F32D-42E6-A0A0-D8271B3F9C1D}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" activeTab="2" xr2:uid="{34119B0E-F32D-42E6-A0A0-D8271B3F9C1D}"/>
   </bookViews>
   <sheets>
     <sheet name="GLORIA to ISIC concordance" sheetId="1" r:id="rId1"/>
@@ -17755,10 +17755,10 @@
         <v>1</v>
       </c>
       <c r="Q101" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R101" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S101" s="8">
         <v>0</v>

</xml_diff>